<commit_message>
Refresh review inputs and analysis pipeline outputs
</commit_message>
<xml_diff>
--- a/outputs/issue_classification_summary.xlsx
+++ b/outputs/issue_classification_summary.xlsx
@@ -443,10 +443,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3018</v>
+        <v>3254</v>
       </c>
       <c r="C2" t="n">
-        <v>53.17</v>
+        <v>52.83</v>
       </c>
     </row>
     <row r="3">
@@ -456,10 +456,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>849</v>
+        <v>927</v>
       </c>
       <c r="C3" t="n">
-        <v>14.96</v>
+        <v>15.05</v>
       </c>
     </row>
     <row r="4">
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>458</v>
+        <v>525</v>
       </c>
       <c r="C4" t="n">
-        <v>8.07</v>
+        <v>8.52</v>
       </c>
     </row>
     <row r="5">
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>378</v>
+        <v>402</v>
       </c>
       <c r="C5" t="n">
-        <v>6.66</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="6">
@@ -495,10 +495,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>354</v>
+        <v>391</v>
       </c>
       <c r="C6" t="n">
-        <v>6.24</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="7">
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="C7" t="n">
-        <v>4.35</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="8">
@@ -521,10 +521,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="C8" t="n">
-        <v>3.7</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="9">
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C9" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="10">
@@ -547,10 +547,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C10" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="11">
@@ -560,10 +560,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C11" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
     </row>
   </sheetData>
@@ -681,34 +681,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="F3" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="G3" t="n">
         <v>11</v>
       </c>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I3" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="J3" t="n">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -718,34 +718,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E4" t="n">
-        <v>342</v>
+        <v>366</v>
       </c>
       <c r="F4" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="G4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H4" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="I4" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J4" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="K4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -761,25 +761,25 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E5" t="n">
-        <v>825</v>
+        <v>842</v>
       </c>
       <c r="F5" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G5" t="n">
         <v>66</v>
       </c>
       <c r="H5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="I5" t="n">
         <v>103</v>
       </c>
       <c r="J5" t="n">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="K5" t="n">
         <v>25</v>
@@ -792,34 +792,34 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
         <v>3</v>
       </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>359</v>
+        <v>455</v>
       </c>
       <c r="F6" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="G6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H6" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I6" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="J6" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
         <v>5</v>
@@ -838,25 +838,25 @@
         <v>45</v>
       </c>
       <c r="E7" t="n">
-        <v>771</v>
+        <v>818</v>
       </c>
       <c r="F7" t="n">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="G7" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H7" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I7" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J7" t="n">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="K7" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merge dates into one column, rebuild pipeline outputs, add Power BI screen
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/issue_classification_summary.xlsx
+++ b/outputs/issue_classification_summary.xlsx
@@ -714,7 +714,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Namma Veedu Vasanta Bhavan</t>
+          <t>Namma Veedu Vasantha Bhavan</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1258,7 +1258,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Namma Veedu Vasanta Bhavan</t>
+          <t>Namma Veedu Vasantha Bhavan</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1278,7 +1278,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Namma Veedu Vasanta Bhavan</t>
+          <t>Namma Veedu Vasantha Bhavan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">

</xml_diff>